<commit_message>
Add practice login test, Excel MCP config, and scope restriction for Excel agent
</commit_message>
<xml_diff>
--- a/test-results.xlsx
+++ b/test-results.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4B6464-E082-4240-8C79-2C8A83939EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Test Results" state="visible" r:id="rId4"/>
+    <sheet name="Practice Login Results" sheetId="2" r:id="rId1"/>
+    <sheet name="Test Results" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>Test Case Name</t>
   </si>
@@ -19,33 +24,101 @@
     <t>Status</t>
   </si>
   <si>
-    <t>logo is visible on homepage</t>
-  </si>
-  <si>
-    <t>Passed</t>
+    <t>search for Claude AI</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Error/Notes</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>5s</t>
+  </si>
+  <si>
+    <t>Google bot detection - redirected to CAPTCHA page (/sorry/index)</t>
+  </si>
+  <si>
+    <t>practicetestautomation login with valid credentials</t>
+  </si>
+  <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t>16s</t>
+  </si>
+  <si>
+    <t>none</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF276221"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -59,7 +132,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,10 +166,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,32 +514,420 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B88E0BC-FB63-4871-98F5-6C436C722B75}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="1" max="1" width="50.6328125" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46155</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E100"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="40.6328125" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" customWidth="1"/>
+    <col min="4" max="4" width="55.6328125" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E5" s="5"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E26" s="5"/>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E28" s="5"/>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E29" s="5"/>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E30" s="5"/>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E31" s="5"/>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E32" s="5"/>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E35" s="5"/>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E37" s="5"/>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E38" s="5"/>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E40" s="5"/>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E41" s="5"/>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E44" s="5"/>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E45" s="5"/>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E47" s="5"/>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E48" s="5"/>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E49" s="5"/>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E50" s="5"/>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E51" s="5"/>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E52" s="5"/>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E53" s="5"/>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E54" s="5"/>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E55" s="5"/>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E56" s="5"/>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E57" s="5"/>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E58" s="5"/>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E59" s="5"/>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E60" s="5"/>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E61" s="5"/>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E62" s="5"/>
+    </row>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E63" s="5"/>
+    </row>
+    <row r="64" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E64" s="5"/>
+    </row>
+    <row r="65" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E65" s="5"/>
+    </row>
+    <row r="66" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E66" s="5"/>
+    </row>
+    <row r="67" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E67" s="5"/>
+    </row>
+    <row r="68" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E68" s="5"/>
+    </row>
+    <row r="69" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E69" s="5"/>
+    </row>
+    <row r="70" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E70" s="5"/>
+    </row>
+    <row r="71" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E71" s="5"/>
+    </row>
+    <row r="72" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E72" s="5"/>
+    </row>
+    <row r="73" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E73" s="5"/>
+    </row>
+    <row r="74" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E74" s="5"/>
+    </row>
+    <row r="75" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E75" s="5"/>
+    </row>
+    <row r="76" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E76" s="5"/>
+    </row>
+    <row r="77" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E77" s="5"/>
+    </row>
+    <row r="78" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E78" s="5"/>
+    </row>
+    <row r="79" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E79" s="5"/>
+    </row>
+    <row r="80" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E80" s="5"/>
+    </row>
+    <row r="81" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E81" s="5"/>
+    </row>
+    <row r="82" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E82" s="5"/>
+    </row>
+    <row r="83" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E83" s="5"/>
+    </row>
+    <row r="84" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E84" s="5"/>
+    </row>
+    <row r="85" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E85" s="5"/>
+    </row>
+    <row r="86" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E86" s="5"/>
+    </row>
+    <row r="87" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E87" s="5"/>
+    </row>
+    <row r="88" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E88" s="5"/>
+    </row>
+    <row r="89" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E89" s="5"/>
+    </row>
+    <row r="90" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E90" s="5"/>
+    </row>
+    <row r="91" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E91" s="5"/>
+    </row>
+    <row r="92" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E92" s="5"/>
+    </row>
+    <row r="93" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E93" s="5"/>
+    </row>
+    <row r="94" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E94" s="5"/>
+    </row>
+    <row r="95" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E95" s="5"/>
+    </row>
+    <row r="96" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E96" s="5"/>
+    </row>
+    <row r="97" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E97" s="5"/>
+    </row>
+    <row r="98" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E98" s="5"/>
+    </row>
+    <row r="99" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E99" s="5"/>
+    </row>
+    <row r="100" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E100" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{549ac42a-3eb4-4074-b885-aea26bd6241e}" enabled="1" method="Standard" siteId="{9274ee3f-9425-4109-a27f-9fb15c10675d}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>